<commit_message>
feat: Add a new workflow for generating scientifically accurate TikTok carousel images of dinosaurs.
</commit_message>
<xml_diff>
--- a/plantilla_dinosaurios_100.xlsx
+++ b/plantilla_dinosaurios_100.xlsx
@@ -2229,7 +2229,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2245,9 +2245,23 @@
         <v>Fecha</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Gigantes del Mar (Que NO son Dinos)</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Pendiente</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2026-02-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Require exact SIZE and update carousel workflow
Add a mandatory 'DIMENSIONS EXACTAS' note to the dinosaur skill (SKILL.md) and revise the carousel workflow: rename Slide 1 to 'Portada/Hook', add a SIZE column to the prompts table (with example entries), and clarify slide naming and content. Also add a new temp_ideas.json with proposed video ideas, and update various output assets (output_ideas.json, plantilla XLSX, tiktok_debug.png, tiktok_profile_data.json) with refreshed data and media.
</commit_message>
<xml_diff>
--- a/plantilla_dinosaurios_100.xlsx
+++ b/plantilla_dinosaurios_100.xlsx
@@ -2217,7 +2217,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2233,20 +2233,6 @@
         <v>Fecha</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Gigantes del Mar (Que NO son Dinos)</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Hecho</v>
-      </c>
-      <c r="D2" t="str">
-        <v>2026-02-01</v>
-      </c>
-    </row>
     <row r="3">
       <c r="A3">
         <v>2</v>
@@ -2303,10 +2289,24 @@
         <v>2026-02-15</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7" t="str">
+        <v>¿Mitos de Película?: Lo que Jurassic Park nos ocultó</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Pendiente</v>
+      </c>
+      <c r="D7" t="str">
+        <v>2026-02-17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7007874015748032" right="0.7007874015748032" top="0.7519685039370079" bottom="0.7519685039370079" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rename 'Dinosaurios' column to 'Dinos Par1' and accept animals
Update manage_ideas.js to use the new column name 'Dinos Par1' when creating the sheet and when appending new ideas. Adjust the workflow docs (carrusel-tiktok-dinos.md) to instruct saving the selected idea along with the animals used and update the example CLI invocation to include an animal list. Also include an updated spreadsheet template (plantilla_dinosaurios_100.xlsx). These changes align the code, docs, and template to store animals alongside ideas.
</commit_message>
<xml_diff>
--- a/plantilla_dinosaurios_100.xlsx
+++ b/plantilla_dinosaurios_100.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="157">
   <si>
     <t>ID</t>
   </si>
@@ -471,13 +471,28 @@
     <t xml:space="preserve">Garras de Pesadilla: Los 7 Dinosaurios con Garras Más Enormes</t>
   </si>
   <si>
+    <t>2026-02-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Therizinosaurus, Deinocheirus, Megaraptor, Utahraptor, Baryonyx, Balaur bondoc, Deinonychus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parásitos de Dinosaurios (Los verdaderos sobrevivientes)</t>
+  </si>
+  <si>
     <t>Pendiente</t>
   </si>
   <si>
-    <t>2026-02-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Therizinosaurus, Deinocheirus, Megaraptor, Utahraptor, Baryonyx, Balaur bondoc, Deinonychus</t>
+    <t>2026-02-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pseudopulex,Deinocroton draculi,Burmaculex antiquus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Top 5 Megaraptóridos Más Grandes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maip macrothorax, Aerosteon riocoloradense, Megaraptor namunhuaiquii, Orkoraptor burkei, Tratayenia roxasi</t>
   </si>
 </sst>
 </file>
@@ -2884,7 +2899,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" min="4" max="4" width="19.875"/>
+    <col customWidth="1" min="4" max="4" width="22.625"/>
+    <col customWidth="1" min="5" max="5" width="43.75390625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2962,7 +2978,7 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
         <v>137</v>
@@ -2975,6 +2991,9 @@
       </c>
     </row>
     <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
       <c r="B8" t="s">
         <v>139</v>
       </c>
@@ -2986,6 +3005,9 @@
       </c>
     </row>
     <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
       <c r="B9" t="s">
         <v>141</v>
       </c>
@@ -2997,6 +3019,9 @@
       </c>
     </row>
     <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
       <c r="B10" t="s">
         <v>143</v>
       </c>
@@ -3008,6 +3033,9 @@
       </c>
     </row>
     <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
       <c r="B11" t="s">
         <v>144</v>
       </c>
@@ -3019,6 +3047,9 @@
       </c>
     </row>
     <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
       <c r="B12" t="s">
         <v>145</v>
       </c>
@@ -3030,6 +3061,9 @@
       </c>
     </row>
     <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
       <c r="B13" t="s">
         <v>146</v>
       </c>
@@ -3041,6 +3075,9 @@
       </c>
     </row>
     <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
       <c r="B14" t="s">
         <v>147</v>
       </c>
@@ -3053,19 +3090,53 @@
     </row>
     <row r="15">
       <c r="A15">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
         <v>148</v>
       </c>
       <c r="C15" t="s">
+        <v>129</v>
+      </c>
+      <c r="D15" t="s">
         <v>149</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>150</v>
       </c>
-      <c r="E15" t="s">
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
         <v>151</v>
+      </c>
+      <c r="C16" t="s">
+        <v>152</v>
+      </c>
+      <c r="D16" t="s">
+        <v>153</v>
+      </c>
+      <c r="E16" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>15</v>
+      </c>
+      <c r="B17" t="s">
+        <v>155</v>
+      </c>
+      <c r="C17" t="s">
+        <v>152</v>
+      </c>
+      <c r="D17" t="s">
+        <v>153</v>
+      </c>
+      <c r="E17" t="s">
+        <v>156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add climate/scene guidance; add UTF-8 ideas
Refine dinosaur prompt guidance: add explicit "Clima y Entorno (SCENE)" instructions and seasonal accuracy to .agent/skills/experto-dinosaurios/SKILL.md and .agent/workflows/generar-imagenes-carrusel.md, tighten wording on Atmosphere/Whisk Scene and Style (remove brand mention, update example to anatomically accurate paleoart). Add new temp_ideas_utf8.json containing a UTF-8 encoded list of idea entries. Updated output_ideas.json and plantilla_dinosaurios_100.xlsx (data/asset updates).
</commit_message>
<xml_diff>
--- a/plantilla_dinosaurios_100.xlsx
+++ b/plantilla_dinosaurios_100.xlsx
@@ -2217,7 +2217,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2472,10 +2472,27 @@
         <v>Deinosuchus, Sarcosuchus, Kaprosuchus, Machimosaurus, Dakosaurus</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19">
+        <v>17</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Plumas Rebeldes: Los dinosaurios con abrigos impresionantes</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Pendiente</v>
+      </c>
+      <c r="D19" t="str">
+        <v>2026-03-06</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Yutyrannus, Microraptor, Sinosauropteryx, Gigantoraptor, Deinocheirus</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7007874015748032" right="0.7007874015748032" top="0.7519685039370079" bottom="0.7519685039370079" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update TikTok profile data and media files
Refresh tiktok_profile_data.json with updated follower/like counts and replace recentVideos entries (links, descriptions, and view counts) to reflect latest posts. Also update associated binary assets: plantilla_dinosaurios_100.xlsx and tiktok_debug.png.
</commit_message>
<xml_diff>
--- a/plantilla_dinosaurios_100.xlsx
+++ b/plantilla_dinosaurios_100.xlsx
@@ -2217,7 +2217,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2489,10 +2489,27 @@
         <v>Yutyrannus, Microraptor, Sinosauropteryx, Gigantoraptor, Deinocheirus</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20">
+        <v>18</v>
+      </c>
+      <c r="B20" t="str">
+        <v>El Turno de Noche: Los Cazadores Nocturnos de la Prehistoria</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Pendiente</v>
+      </c>
+      <c r="D20" t="str">
+        <v>2026-04-14</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Stenonychosaurus, Shuvuuia, Juravenator, Velociraptor mongoliensis</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7007874015748032" right="0.7007874015748032" top="0.7519685039370079" bottom="0.7519685039370079" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E20"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>